<commit_message>
Test Cases and implementation of Load Testing
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Non-Functional Testing Suite/Load Tests.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Non-Functional Testing Suite/Load Tests.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="65">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -27,9 +27,6 @@
     <t>Test Case Title</t>
   </si>
   <si>
-    <t>Test Case Type</t>
-  </si>
-  <si>
     <t>Preconditions</t>
   </si>
   <si>
@@ -48,13 +45,175 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>1.</t>
-  </si>
-  <si>
-    <t>2.</t>
-  </si>
-  <si>
-    <t>3.</t>
+    <t>Status (Mobile)</t>
+  </si>
+  <si>
+    <t>TC-LD-1</t>
+  </si>
+  <si>
+    <t>Login Time</t>
+  </si>
+  <si>
+    <t>Verification of loading time for such pages as: login, entering password processing and logout</t>
+  </si>
+  <si>
+    <t>1. Enter Amazon main page                                                                2. Manage registration or Login to account processes</t>
+  </si>
+  <si>
+    <t>2. Login and measure time for this action</t>
+  </si>
+  <si>
+    <t>3. Enter password and measure time for this action</t>
+  </si>
+  <si>
+    <t>1. Logout and measure the time for this action</t>
+  </si>
+  <si>
+    <t>The time of all processes must not take longer than 1.5-2 seconds</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>All test cases included next load tests activities were repeted 3 times</t>
+  </si>
+  <si>
+    <t>TC-LD-2</t>
+  </si>
+  <si>
+    <t>Product Page</t>
+  </si>
+  <si>
+    <t>1. Enter Amazon main page                                                                2. Choose any product (face mask)</t>
+  </si>
+  <si>
+    <t>Verification of loading time for product pages (changing size, colour, and products)</t>
+  </si>
+  <si>
+    <t>1. Measure the time for product page loading</t>
+  </si>
+  <si>
+    <t>The time of all processes must not take longer than 2 seconds</t>
+  </si>
+  <si>
+    <t>2. Provide different changes of the product</t>
+  </si>
+  <si>
+    <t>3. Measure time and check with other products</t>
+  </si>
+  <si>
+    <t>TC-LD-3</t>
+  </si>
+  <si>
+    <t>Product Searching</t>
+  </si>
+  <si>
+    <t>Product Filtering</t>
+  </si>
+  <si>
+    <t>TC-LD-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter Amazon main page                                                               </t>
+  </si>
+  <si>
+    <t>Verification of loading time for product searching</t>
+  </si>
+  <si>
+    <t>1. Enter the name of a product and check the load time</t>
+  </si>
+  <si>
+    <t>2. Enter the invalid name of a product and check the load time</t>
+  </si>
+  <si>
+    <t>3. Repeat the processes with other products</t>
+  </si>
+  <si>
+    <t>The time of all processes must not take longer than 2.5 seconds</t>
+  </si>
+  <si>
+    <t>1. Enter Amazon main page                                                                2. Enter the name of product (rat toy)</t>
+  </si>
+  <si>
+    <t>Verification of loading time for product pages after filtering</t>
+  </si>
+  <si>
+    <t>1. Measure the time for products list page loading</t>
+  </si>
+  <si>
+    <t>2. Provide different filtering changes (price, brands, species)</t>
+  </si>
+  <si>
+    <t>3. Measure time and check with other filter processes</t>
+  </si>
+  <si>
+    <t>Cart Management 1</t>
+  </si>
+  <si>
+    <t>TC-LD-5</t>
+  </si>
+  <si>
+    <t>Cart Management 2</t>
+  </si>
+  <si>
+    <t>Cart Management 3</t>
+  </si>
+  <si>
+    <t>1. Enter Amazon main page                                                                2. Choose any product (rabbit plush toy)</t>
+  </si>
+  <si>
+    <t>Verification of loading time for adding product to the cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click on "Add to Cart" button </t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Repeat up to 3 times with this and other products </t>
+  </si>
+  <si>
+    <t>The time of all processes must not take longer than 1.5 seconds</t>
+  </si>
+  <si>
+    <t>TC-LD-6</t>
+  </si>
+  <si>
+    <t>TC-LD-7</t>
+  </si>
+  <si>
+    <t>1. Enter Amazon main page                                                                2. Make the TC-LD-5</t>
+  </si>
+  <si>
+    <t>Verification of loading time for opening the cart</t>
+  </si>
+  <si>
+    <t>2. Measure time for the process</t>
+  </si>
+  <si>
+    <t>1. Open the Cart with product and easure time for the process</t>
+  </si>
+  <si>
+    <t>2. Leave the Cart page and repeat up to 3 times</t>
+  </si>
+  <si>
+    <t>3. Can be providen after TC-LD-7 with empty cart</t>
+  </si>
+  <si>
+    <t>1. Enter Amazon main page                                                                2. Make the TC-LD-5 and TC-LD-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verification of loading time for deleting </t>
+  </si>
+  <si>
+    <t>Time for loading the empty cart is about the same as with cart with several products</t>
+  </si>
+  <si>
+    <t>1. Delete the product from cart and check the time</t>
+  </si>
+  <si>
+    <t>2. Repeat with other products</t>
+  </si>
+  <si>
+    <t>3. Repeat after TC-LD-5 and TC-LD-6 again</t>
   </si>
 </sst>
 </file>
@@ -142,18 +301,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,17 +608,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" customWidth="1"/>
-    <col min="9" max="9" width="10.109375" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="4" max="4" width="27.44140625" customWidth="1"/>
+    <col min="5" max="5" width="53.109375" customWidth="1"/>
+    <col min="6" max="6" width="28.5546875" customWidth="1"/>
+    <col min="7" max="7" width="7.77734375" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" customWidth="1"/>
+    <col min="9" max="9" width="31" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -471,61 +646,445 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="8"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="8"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="9"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="9"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="7"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="8"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="9"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="7"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="8"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="9"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="9"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="7"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="9"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="9"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" s="7"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="8"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="9"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="9"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F18" s="8"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="8"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F19" s="9"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="9"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F21" s="8"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="8"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F22" s="9"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="56">
+    <mergeCell ref="G17:G19"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="F20:F22"/>
+    <mergeCell ref="G20:G22"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="I20:I22"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="G11:G13"/>
+    <mergeCell ref="H11:H13"/>
+    <mergeCell ref="I11:I13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="C14:C16"/>
+    <mergeCell ref="D14:D16"/>
+    <mergeCell ref="F14:F16"/>
+    <mergeCell ref="G14:G16"/>
+    <mergeCell ref="H14:H16"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="D11:D13"/>
+    <mergeCell ref="F11:F13"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="G2:G4"/>
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="I2:I4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="F2:F4"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="I2:I4"/>
-    <mergeCell ref="G2:G4"/>
-    <mergeCell ref="H2:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>